<commit_message>
Mod8 Exer 3 incomplete MySQL Blog DB 101.docx
</commit_message>
<xml_diff>
--- a/module8/exercise1/blog_pdm.xlsx
+++ b/module8/exercise1/blog_pdm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/408a8262ffb9e406/organisedshare.ai/Institute of Data/2026-02-02-SE-FT-AP-A-B/institute-of-data-labs/module8/exercise1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_1BC18C055640080D106E8CF2515ED87656CD5A63" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92D10AF1-48FB-4528-9953-A16909A4A201}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="11_1BC18C055640080D106E8CF2515ED87656CD5A63" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78A728AE-A1B2-4E43-8A62-8CFB79D07958}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="108">
   <si>
     <t>BLOG - PHYSICAL DATA MODEL</t>
   </si>
@@ -395,12 +395,72 @@
       <t>Foreign Key (FK) is:</t>
     </r>
   </si>
+  <si>
+    <t>THIS IS V IMPORTANT</t>
+  </si>
+  <si>
+    <t>A whole number (no decimals). Perfect for IDs and counts. e.g. 1, 42, 1000</t>
+  </si>
+  <si>
+    <t>Variable-length text, max 50 characters. 'VARCHAR' = Variable Character. Use for short text like names.</t>
+  </si>
+  <si>
+    <t>Variable-length text, max 100 characters. Same as VARCHAR(50) but allows longer text — good for email addresses.</t>
+  </si>
+  <si>
+    <t>Stores a date + time together (e.g. '2024-06-15 10:30:00'). Auto-records when a row was created/updated.</t>
+  </si>
+  <si>
+    <t>A whole number. Used here as a Foreign Key — it stores the user_id of whoever wrote the post.</t>
+  </si>
+  <si>
+    <t>Variable-length text, max 200 characters. Enough room for a typical blog post title.</t>
+  </si>
+  <si>
+    <t>Unlimited-length text. No character limit — ideal for long blog post content/body.</t>
+  </si>
+  <si>
+    <t>Variable-length text, max 255 characters. Stores a web link (URL) to an image. 255 is a common max URL length.</t>
+  </si>
+  <si>
+    <t>Stores a date + time. Records when the post was first created.</t>
+  </si>
+  <si>
+    <t>Stores a date + time. Automatically refreshes to the current time whenever the post row is edited.</t>
+  </si>
+  <si>
+    <t>A whole number. Foreign Key pointing to the comments table — identifies which comment this is.</t>
+  </si>
+  <si>
+    <t>A whole number. Foreign Key — stores the post_id of the post being commented on.</t>
+  </si>
+  <si>
+    <t>A whole number. Foreign Key — stores the user_id of the user who wrote the comment.</t>
+  </si>
+  <si>
+    <t>Unlimited-length text. Stores the full text of the comment.</t>
+  </si>
+  <si>
+    <t>Stores a date + time. Records when the comment was posted.</t>
+  </si>
+  <si>
+    <t>A whole number. Foreign Key — identifies which user gave the like. Together with post_id, forms the Primary Key.</t>
+  </si>
+  <si>
+    <t>A whole number. Foreign Key — identifies which post was liked. Together with user_id, forms the Primary Key.</t>
+  </si>
+  <si>
+    <t>Stores a date + time. Records the exact moment the like was given.</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,6 +528,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -510,30 +585,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -546,6 +615,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,6 +640,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -846,572 +929,664 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{0BD6B289-30F9-4529-AC07-E363D8C96990}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="15" style="3" customWidth="1"/>
-    <col min="4" max="4" width="50" style="3" customWidth="1"/>
-    <col min="5" max="5" width="45" style="3" customWidth="1"/>
-    <col min="6" max="7" width="5" style="3" customWidth="1"/>
-    <col min="8" max="11" width="9.140625" style="3"/>
-    <col min="12" max="12" width="80.85546875" style="3" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" customWidth="1"/>
+    <col min="4" max="4" width="85.42578125" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="45" customWidth="1"/>
+    <col min="7" max="8" width="5" customWidth="1"/>
+    <col min="13" max="13" width="80.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="3" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+    </row>
+    <row r="3" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C4" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="G5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="H5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="M5" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="L6" s="9"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7" t="s">
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="M6" s="5"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="L7" s="12" t="s">
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="M7" s="8" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="L8" s="12" t="s">
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="M8" s="8" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7" t="s">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="L9" s="12" t="s">
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="M9" s="8" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L10" s="12" t="s">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D10" s="16"/>
+      <c r="M10" s="8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="F11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7" t="s">
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="4"/>
+      <c r="H12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L12" s="11" t="s">
+      <c r="M12" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7" t="s">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="F13" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="L13" s="9"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7" t="s">
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="M13" s="5"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7" t="s">
+      <c r="D14" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="L14" s="13" t="s">
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="M14" s="9" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7" t="s">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7" t="s">
+      <c r="D15" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="L15" s="13" t="s">
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="M15" s="9" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7" t="s">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="F16" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="L16" s="13" t="s">
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="M16" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7" t="s">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="L17" s="13" t="s">
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="M17" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L18" s="13" t="s">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D18" s="16"/>
+      <c r="M18" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="F19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7" t="s">
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="F20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="4"/>
+      <c r="H20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L20" s="11" t="s">
+      <c r="M20" s="7" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7" t="s">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="4"/>
+      <c r="H21" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L21" s="13"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7" t="s">
+      <c r="M21" s="9"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="F22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="L22" s="13" t="s">
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="M22" s="9" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7" t="s">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="F23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="L23" s="13" t="s">
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="M23" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L24" s="13" t="s">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D24" s="16"/>
+      <c r="M24" s="9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="4"/>
+      <c r="H25" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L25" s="13"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7" t="s">
+      <c r="M25" s="9"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="F26" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="4"/>
+      <c r="H26" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L26" s="11" t="s">
+      <c r="M26" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7" t="s">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="F27" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="L27" s="11"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L28" s="14" t="s">
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="M27" s="7"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M28" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L29" s="14" t="s">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M29" s="10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-    </row>
-    <row r="32" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="D33" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="E33" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="D34" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="E34" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L34" s="6"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+      <c r="M34" s="2"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="D35" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="E35" s="6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="D36" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="E36" s="6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="D37" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="E37" s="6" t="s">
         <v>69</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>